<commit_message>
Dati: risultati quarti + accoppiamenti semifinali (mar 14/07)
- Quarti giocati: I Cugini 15-7 Gli Allenati, Gli Zebis 12-5 Gli Hummarell,
  Bad Boys 12-6 Chocolate Starfishes, Lord&Chri 12-3 Ricci di Mare
- Semifinali (mar 14/07): I Cugini vs Gli Zebis (20:45),
  Bad Boys vs Lord&Chri (21:30)
- Finale: orari aggiornati (ven 17/07 21:00 e 21:45)
- Check campo unico: nessuna sovrapposizione

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026.xlsx
+++ b/Resources/Calend Bocce 2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="241">
   <si>
     <t>data e ora</t>
   </si>
@@ -394,16 +394,22 @@
     <t>QUAR4</t>
   </si>
   <si>
+    <t>martedì 14/07 20:45</t>
+  </si>
+  <si>
     <t>SEMI</t>
   </si>
   <si>
-    <t>venerdì 17/07 20:45</t>
+    <t>martedì 14/07 21:30</t>
+  </si>
+  <si>
+    <t>venerdì 17/07 21:00</t>
   </si>
   <si>
     <t>FIN 3°</t>
   </si>
   <si>
-    <t>venerdì 17/07 21:30</t>
+    <t>venerdì 17/07 21:45</t>
   </si>
   <si>
     <t>FIN 1°</t>
@@ -737,7 +743,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -790,10 +796,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -913,7 +915,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="88">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1042,40 +1044,37 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="10" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="10" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="11" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="9" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1129,16 +1128,16 @@
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="12" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="12" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -2698,56 +2697,92 @@
       <c r="D79" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="E79" s="50"/>
-      <c r="F79" s="50"/>
+      <c r="E79" s="46">
+        <v>6.0</v>
+      </c>
+      <c r="F79" s="46">
+        <v>8.0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B80" s="51" t="s">
+      <c r="B80" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="C80" s="45"/>
-      <c r="D80" s="48"/>
-      <c r="E80" s="52"/>
-      <c r="F80" s="52"/>
+      <c r="C80" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D80" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="E80" s="46">
+        <v>15.0</v>
+      </c>
+      <c r="F80" s="46">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B81" s="51" t="s">
+      <c r="B81" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="C81" s="45"/>
-      <c r="D81" s="48"/>
-      <c r="E81" s="52"/>
-      <c r="F81" s="52"/>
+      <c r="C81" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="D81" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="E81" s="46">
+        <v>12.0</v>
+      </c>
+      <c r="F81" s="46">
+        <v>5.0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B82" s="51" t="s">
+      <c r="B82" s="50" t="s">
         <v>123</v>
       </c>
-      <c r="C82" s="48"/>
-      <c r="D82" s="48"/>
-      <c r="E82" s="52"/>
-      <c r="F82" s="52"/>
+      <c r="C82" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="D82" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="E82" s="46">
+        <v>12.0</v>
+      </c>
+      <c r="F82" s="46">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B83" s="51" t="s">
+      <c r="B83" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="C83" s="48"/>
-      <c r="D83" s="48"/>
-      <c r="E83" s="52"/>
-      <c r="F83" s="52"/>
+      <c r="C83" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E83" s="46">
+        <v>12.0</v>
+      </c>
+      <c r="F83" s="46">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="39"/>
@@ -2757,24 +2792,36 @@
       <c r="F84" s="49"/>
     </row>
     <row r="85">
-      <c r="A85" s="5"/>
-      <c r="B85" s="51" t="s">
+      <c r="A85" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C85" s="48"/>
-      <c r="D85" s="48"/>
-      <c r="E85" s="52"/>
-      <c r="F85" s="52"/>
+      <c r="B85" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="C85" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D85" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="E85" s="51"/>
+      <c r="F85" s="51"/>
     </row>
     <row r="86">
-      <c r="A86" s="5"/>
-      <c r="B86" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="C86" s="48"/>
-      <c r="D86" s="48"/>
-      <c r="E86" s="52"/>
-      <c r="F86" s="52"/>
+      <c r="A86" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B86" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="C86" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="D86" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="E86" s="51"/>
+      <c r="F86" s="51"/>
     </row>
     <row r="87">
       <c r="B87" s="39"/>
@@ -2785,10 +2832,10 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B88" s="53" t="s">
-        <v>128</v>
+        <v>129</v>
+      </c>
+      <c r="B88" s="52" t="s">
+        <v>130</v>
       </c>
       <c r="C88" s="48"/>
       <c r="D88" s="48"/>
@@ -2797,10 +2844,10 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B89" s="53" t="s">
-        <v>130</v>
+        <v>131</v>
+      </c>
+      <c r="B89" s="52" t="s">
+        <v>132</v>
       </c>
       <c r="C89" s="48"/>
       <c r="D89" s="48"/>
@@ -9164,54 +9211,54 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="54" t="s">
-        <v>131</v>
-      </c>
-      <c r="B1" s="55" t="s">
-        <v>132</v>
-      </c>
-      <c r="C1" s="56" t="s">
+      <c r="A1" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="D1" s="57" t="s">
+      <c r="B1" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="C1" s="55" t="s">
         <v>135</v>
       </c>
-      <c r="F1" s="59" t="s">
+      <c r="D1" s="56" t="s">
         <v>136</v>
       </c>
-      <c r="G1" s="60" t="s">
+      <c r="E1" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="H1" s="61" t="s">
+      <c r="F1" s="58" t="s">
         <v>138</v>
+      </c>
+      <c r="G1" s="59" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="60" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="61" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="63" t="s">
+      <c r="D2" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="65" t="s">
+      <c r="F2" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="66" t="s">
+      <c r="G2" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="67" t="s">
+      <c r="H2" s="66" t="s">
         <v>23</v>
       </c>
     </row>
@@ -9219,25 +9266,25 @@
       <c r="A3" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="61" t="s">
         <v>67</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="63" t="s">
+      <c r="D3" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="64" t="s">
+      <c r="E3" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="65" t="s">
+      <c r="F3" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="66" t="s">
+      <c r="G3" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="67" t="s">
+      <c r="H3" s="66" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9245,25 +9292,25 @@
       <c r="A4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="61" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="63" t="s">
+      <c r="D4" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="64" t="s">
+      <c r="E4" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="65" t="s">
+      <c r="F4" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="66" t="s">
+      <c r="G4" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="67" t="s">
+      <c r="H4" s="66" t="s">
         <v>24</v>
       </c>
     </row>
@@ -9271,22 +9318,22 @@
       <c r="A5" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="61" t="s">
         <v>40</v>
       </c>
       <c r="C5" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="64" t="s">
+      <c r="E5" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="65" t="s">
+      <c r="F5" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="66" t="s">
+      <c r="G5" s="65" t="s">
         <v>38</v>
       </c>
       <c r="H5" s="11" t="s">
@@ -9294,8 +9341,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="68"/>
-      <c r="B6" s="68"/>
+      <c r="A6" s="67"/>
+      <c r="B6" s="67"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
@@ -9339,25 +9386,25 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="69" t="s">
+      <c r="E1" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="69" t="s">
+      <c r="F1" s="68" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="4"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B2" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="B2" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="70" t="s">
+      <c r="D2" s="69" t="s">
         <v>59</v>
       </c>
       <c r="E2" s="46">
@@ -9369,16 +9416,16 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B3" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C3" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="D3" s="71" t="s">
+      <c r="B3" s="70" t="s">
         <v>144</v>
+      </c>
+      <c r="C3" s="70" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="70" t="s">
+        <v>146</v>
       </c>
       <c r="E3" s="46">
         <v>9.0</v>
@@ -9389,15 +9436,15 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B4" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C4" s="72" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="72" t="s">
+      <c r="B4" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="71" t="s">
+        <v>149</v>
+      </c>
+      <c r="D4" s="71" t="s">
         <v>40</v>
       </c>
       <c r="E4" s="46">
@@ -9409,16 +9456,16 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B5" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C5" s="73" t="s">
         <v>150</v>
       </c>
-      <c r="D5" s="73" t="s">
+      <c r="B5" s="72" t="s">
         <v>151</v>
+      </c>
+      <c r="C5" s="72" t="s">
+        <v>152</v>
+      </c>
+      <c r="D5" s="72" t="s">
+        <v>153</v>
       </c>
       <c r="E5" s="46">
         <v>11.0</v>
@@ -9429,16 +9476,16 @@
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="B6" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C6" s="74" t="s">
         <v>154</v>
       </c>
-      <c r="D6" s="74" t="s">
+      <c r="B6" s="73" t="s">
         <v>155</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>156</v>
+      </c>
+      <c r="D6" s="73" t="s">
+        <v>157</v>
       </c>
       <c r="E6" s="46">
         <v>4.0</v>
@@ -9450,16 +9497,16 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C7" s="73" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="73" t="s">
-        <v>157</v>
+      <c r="D7" s="72" t="s">
+        <v>159</v>
       </c>
       <c r="E7" s="46">
         <v>11.0</v>
@@ -9470,21 +9517,21 @@
     </row>
     <row r="8">
       <c r="A8" s="20"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="B9" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9" s="73" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="73" t="s">
-        <v>150</v>
+      <c r="D9" s="72" t="s">
+        <v>152</v>
       </c>
       <c r="E9" s="46">
         <v>6.0</v>
@@ -9495,15 +9542,15 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="B10" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="70" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="70" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C10" s="69" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="69" t="s">
         <v>21</v>
       </c>
       <c r="E10" s="46">
@@ -9516,16 +9563,16 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B11" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C11" s="71" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="70" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="71" t="s">
-        <v>162</v>
+      <c r="D11" s="70" t="s">
+        <v>164</v>
       </c>
       <c r="E11" s="46">
         <v>10.0</v>
@@ -9536,15 +9583,15 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="B12" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C12" s="70" t="s">
-        <v>164</v>
-      </c>
-      <c r="D12" s="70" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="69" t="s">
+        <v>166</v>
+      </c>
+      <c r="D12" s="69" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="46">
@@ -9555,17 +9602,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="76" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C13" s="74" t="s">
+      <c r="A13" s="75" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="74" t="s">
-        <v>166</v>
+      <c r="D13" s="73" t="s">
+        <v>168</v>
       </c>
       <c r="E13" s="46">
         <v>6.0</v>
@@ -9576,15 +9623,15 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B14" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C14" s="77" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="C14" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="77" t="s">
+      <c r="D14" s="76" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="46">
@@ -9603,16 +9650,16 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B16" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C16" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="B16" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="C16" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="77" t="s">
-        <v>170</v>
+      <c r="D16" s="76" t="s">
+        <v>172</v>
       </c>
       <c r="E16" s="46">
         <v>8.0</v>
@@ -9623,16 +9670,16 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="B17" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C17" s="73" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C17" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="73" t="s">
-        <v>151</v>
+      <c r="D17" s="72" t="s">
+        <v>153</v>
       </c>
       <c r="E17" s="46">
         <v>7.0</v>
@@ -9643,16 +9690,16 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B18" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C18" s="72" t="s">
+        <v>174</v>
+      </c>
+      <c r="B18" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C18" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="72" t="s">
-        <v>173</v>
+      <c r="D18" s="71" t="s">
+        <v>175</v>
       </c>
       <c r="E18" s="46">
         <v>7.0</v>
@@ -9663,16 +9710,16 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B19" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C19" s="73" t="s">
+        <v>176</v>
+      </c>
+      <c r="B19" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C19" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="73" t="s">
-        <v>150</v>
+      <c r="D19" s="72" t="s">
+        <v>152</v>
       </c>
       <c r="E19" s="46">
         <v>9.0</v>
@@ -9683,16 +9730,16 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B20" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C20" s="72" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="72" t="s">
-        <v>176</v>
+        <v>177</v>
+      </c>
+      <c r="B20" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C20" s="71" t="s">
+        <v>149</v>
+      </c>
+      <c r="D20" s="71" t="s">
+        <v>178</v>
       </c>
       <c r="E20" s="46">
         <v>6.0</v>
@@ -9703,16 +9750,16 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="B21" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C21" s="72" t="s">
+        <v>179</v>
+      </c>
+      <c r="B21" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="71" t="s">
+        <v>180</v>
+      </c>
+      <c r="D21" s="71" t="s">
         <v>178</v>
-      </c>
-      <c r="D21" s="72" t="s">
-        <v>176</v>
       </c>
       <c r="E21" s="46">
         <v>7.0</v>
@@ -9728,32 +9775,32 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="B23" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C23" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D23" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E23" s="79"/>
-      <c r="F23" s="79"/>
+        <v>181</v>
+      </c>
+      <c r="B23" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D23" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C24" s="71" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="70" t="s">
         <v>144</v>
       </c>
-      <c r="D24" s="71" t="s">
-        <v>162</v>
+      <c r="C24" s="70" t="s">
+        <v>146</v>
+      </c>
+      <c r="D24" s="70" t="s">
+        <v>164</v>
       </c>
       <c r="E24" s="46">
         <v>5.0</v>
@@ -9764,15 +9811,15 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B25" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C25" s="70" t="s">
-        <v>164</v>
-      </c>
-      <c r="D25" s="70" t="s">
+        <v>184</v>
+      </c>
+      <c r="B25" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="69" t="s">
+        <v>166</v>
+      </c>
+      <c r="D25" s="69" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="46">
@@ -9784,16 +9831,16 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="B26" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C26" s="72" t="s">
-        <v>147</v>
-      </c>
-      <c r="D26" s="72" t="s">
-        <v>178</v>
+        <v>185</v>
+      </c>
+      <c r="B26" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C26" s="71" t="s">
+        <v>149</v>
+      </c>
+      <c r="D26" s="71" t="s">
+        <v>180</v>
       </c>
       <c r="E26" s="46">
         <v>8.0</v>
@@ -9803,17 +9850,17 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="76" t="s">
-        <v>184</v>
-      </c>
-      <c r="B27" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C27" s="74" t="s">
-        <v>154</v>
-      </c>
-      <c r="D27" s="74" t="s">
-        <v>166</v>
+      <c r="A27" s="75" t="s">
+        <v>186</v>
+      </c>
+      <c r="B27" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="C27" s="73" t="s">
+        <v>156</v>
+      </c>
+      <c r="D27" s="73" t="s">
+        <v>168</v>
       </c>
       <c r="E27" s="46">
         <v>8.0</v>
@@ -9823,17 +9870,17 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="76" t="s">
-        <v>185</v>
-      </c>
-      <c r="B28" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C28" s="74" t="s">
+      <c r="A28" s="75" t="s">
+        <v>187</v>
+      </c>
+      <c r="B28" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="C28" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="74" t="s">
-        <v>155</v>
+      <c r="D28" s="73" t="s">
+        <v>157</v>
       </c>
       <c r="E28" s="46">
         <v>9.0</v>
@@ -9849,15 +9896,15 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B30" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C30" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="D30" s="71" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" s="70" t="s">
+        <v>144</v>
+      </c>
+      <c r="C30" s="70" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="70" t="s">
         <v>37</v>
       </c>
       <c r="E30" s="46">
@@ -9869,16 +9916,16 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="B31" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C31" s="73" t="s">
+        <v>189</v>
+      </c>
+      <c r="B31" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C31" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="73" t="s">
-        <v>151</v>
+      <c r="D31" s="72" t="s">
+        <v>153</v>
       </c>
       <c r="E31" s="46">
         <v>5.0</v>
@@ -9889,16 +9936,16 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B32" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C32" s="72" t="s">
+        <v>190</v>
+      </c>
+      <c r="B32" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="72" t="s">
-        <v>176</v>
+      <c r="D32" s="71" t="s">
+        <v>178</v>
       </c>
       <c r="E32" s="46">
         <v>5.0</v>
@@ -9909,15 +9956,15 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="B33" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C33" s="77" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="77" t="s">
+      <c r="D33" s="76" t="s">
         <v>51</v>
       </c>
       <c r="E33" s="46">
@@ -9929,16 +9976,16 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="B34" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C34" s="73" t="s">
-        <v>150</v>
-      </c>
-      <c r="D34" s="73" t="s">
-        <v>157</v>
+        <v>192</v>
+      </c>
+      <c r="B34" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C34" s="72" t="s">
+        <v>152</v>
+      </c>
+      <c r="D34" s="72" t="s">
+        <v>159</v>
       </c>
       <c r="E34" s="46">
         <v>9.0</v>
@@ -9949,16 +9996,16 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="B35" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C35" s="77" t="s">
+        <v>193</v>
+      </c>
+      <c r="B35" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="C35" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="77" t="s">
-        <v>170</v>
+      <c r="D35" s="76" t="s">
+        <v>172</v>
       </c>
       <c r="E35" s="46">
         <v>2.0</v>
@@ -9974,32 +10021,32 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="B37" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C37" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D37" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E37" s="79"/>
-      <c r="F37" s="79"/>
+        <v>194</v>
+      </c>
+      <c r="B37" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D37" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E37" s="78"/>
+      <c r="F37" s="78"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="B38" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C38" s="74" t="s">
-        <v>166</v>
-      </c>
-      <c r="D38" s="74" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" s="73" t="s">
         <v>155</v>
+      </c>
+      <c r="C38" s="73" t="s">
+        <v>168</v>
+      </c>
+      <c r="D38" s="73" t="s">
+        <v>157</v>
       </c>
       <c r="E38" s="46">
         <v>8.0</v>
@@ -10009,16 +10056,16 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="76" t="s">
-        <v>194</v>
-      </c>
-      <c r="B39" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C39" s="77" t="s">
+      <c r="A39" s="75" t="s">
+        <v>196</v>
+      </c>
+      <c r="B39" s="76" t="s">
         <v>170</v>
       </c>
-      <c r="D39" s="77" t="s">
+      <c r="C39" s="76" t="s">
+        <v>172</v>
+      </c>
+      <c r="D39" s="76" t="s">
         <v>51</v>
       </c>
       <c r="E39" s="46">
@@ -10030,16 +10077,16 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="B40" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C40" s="70" t="s">
-        <v>160</v>
-      </c>
-      <c r="D40" s="70" t="s">
-        <v>164</v>
+        <v>197</v>
+      </c>
+      <c r="B40" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C40" s="69" t="s">
+        <v>162</v>
+      </c>
+      <c r="D40" s="69" t="s">
+        <v>166</v>
       </c>
       <c r="E40" s="46">
         <v>1.0</v>
@@ -10050,15 +10097,15 @@
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="B41" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C41" s="71" t="s">
+        <v>198</v>
+      </c>
+      <c r="B41" s="70" t="s">
         <v>144</v>
       </c>
-      <c r="D41" s="71" t="s">
+      <c r="C41" s="70" t="s">
+        <v>146</v>
+      </c>
+      <c r="D41" s="70" t="s">
         <v>37</v>
       </c>
       <c r="E41" s="46">
@@ -10070,19 +10117,19 @@
     </row>
     <row r="42">
       <c r="A42" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="B42" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C42" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D42" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E42" s="79"/>
-      <c r="F42" s="79"/>
+        <v>199</v>
+      </c>
+      <c r="B42" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C42" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D42" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
     </row>
     <row r="43">
       <c r="A43" s="20"/>
@@ -10091,48 +10138,48 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B44" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C44" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D44" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E44" s="79"/>
-      <c r="F44" s="79"/>
+        <v>200</v>
+      </c>
+      <c r="B44" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C44" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D44" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="B45" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C45" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D45" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E45" s="79"/>
-      <c r="F45" s="79"/>
+        <v>201</v>
+      </c>
+      <c r="B45" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D45" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E45" s="78"/>
+      <c r="F45" s="78"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B46" s="74" t="s">
-        <v>153</v>
-      </c>
-      <c r="C46" s="74" t="s">
+        <v>202</v>
+      </c>
+      <c r="B46" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="C46" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="74" t="s">
-        <v>154</v>
+      <c r="D46" s="73" t="s">
+        <v>156</v>
       </c>
       <c r="E46" s="46">
         <v>7.0</v>
@@ -10143,16 +10190,16 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="B47" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C47" s="72" t="s">
-        <v>178</v>
-      </c>
-      <c r="D47" s="72" t="s">
-        <v>173</v>
+        <v>203</v>
+      </c>
+      <c r="B47" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C47" s="71" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" s="71" t="s">
+        <v>175</v>
       </c>
       <c r="E47" s="46">
         <v>4.0</v>
@@ -10163,15 +10210,15 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B48" s="77" t="s">
-        <v>168</v>
-      </c>
-      <c r="C48" s="77" t="s">
+        <v>204</v>
+      </c>
+      <c r="B48" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="C48" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="77" t="s">
+      <c r="D48" s="76" t="s">
         <v>27</v>
       </c>
       <c r="E48" s="46">
@@ -10183,16 +10230,16 @@
     </row>
     <row r="49">
       <c r="A49" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="B49" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C49" s="73" t="s">
+        <v>205</v>
+      </c>
+      <c r="B49" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C49" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="D49" s="73" t="s">
-        <v>157</v>
+      <c r="D49" s="72" t="s">
+        <v>159</v>
       </c>
       <c r="E49" s="46">
         <v>6.0</v>
@@ -10208,99 +10255,99 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="B51" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C51" s="72" t="s">
-        <v>147</v>
-      </c>
-      <c r="D51" s="72" t="s">
-        <v>173</v>
-      </c>
-      <c r="E51" s="79"/>
-      <c r="F51" s="79"/>
+        <v>206</v>
+      </c>
+      <c r="B51" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C51" s="71" t="s">
+        <v>149</v>
+      </c>
+      <c r="D51" s="71" t="s">
+        <v>175</v>
+      </c>
+      <c r="E51" s="78"/>
+      <c r="F51" s="78"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B52" s="71" t="s">
-        <v>142</v>
-      </c>
-      <c r="C52" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="D52" s="71" t="s">
-        <v>162</v>
-      </c>
-      <c r="E52" s="79"/>
-      <c r="F52" s="79"/>
+        <v>207</v>
+      </c>
+      <c r="B52" s="70" t="s">
+        <v>144</v>
+      </c>
+      <c r="C52" s="70" t="s">
+        <v>145</v>
+      </c>
+      <c r="D52" s="70" t="s">
+        <v>164</v>
+      </c>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="B53" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C53" s="72" t="s">
+        <v>208</v>
+      </c>
+      <c r="B53" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C53" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="D53" s="72" t="s">
-        <v>178</v>
-      </c>
-      <c r="E53" s="79"/>
-      <c r="F53" s="79"/>
+      <c r="D53" s="71" t="s">
+        <v>180</v>
+      </c>
+      <c r="E53" s="78"/>
+      <c r="F53" s="78"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B54" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C54" s="73" t="s">
+        <v>209</v>
+      </c>
+      <c r="B54" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="C54" s="72" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="73" t="s">
+      <c r="D54" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="79"/>
-      <c r="F54" s="79"/>
+      <c r="E54" s="78"/>
+      <c r="F54" s="78"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="B55" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C55" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D55" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E55" s="79"/>
-      <c r="F55" s="79"/>
+        <v>210</v>
+      </c>
+      <c r="B55" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C55" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D55" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E55" s="78"/>
+      <c r="F55" s="78"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="B56" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C56" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D56" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E56" s="79"/>
-      <c r="F56" s="79"/>
+        <v>211</v>
+      </c>
+      <c r="B56" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C56" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D56" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E56" s="78"/>
+      <c r="F56" s="78"/>
     </row>
     <row r="57">
       <c r="A57" s="20"/>
@@ -10309,99 +10356,99 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B58" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C58" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D58" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E58" s="79"/>
-      <c r="F58" s="79"/>
+        <v>212</v>
+      </c>
+      <c r="B58" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C58" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D58" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E58" s="78"/>
+      <c r="F58" s="78"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="B59" s="70" t="s">
-        <v>140</v>
-      </c>
-      <c r="C59" s="70" t="s">
-        <v>160</v>
-      </c>
-      <c r="D59" s="70" t="s">
+        <v>213</v>
+      </c>
+      <c r="B59" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59" s="69" t="s">
+        <v>162</v>
+      </c>
+      <c r="D59" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="E59" s="79"/>
-      <c r="F59" s="79"/>
+      <c r="E59" s="78"/>
+      <c r="F59" s="78"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="B60" s="73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C60" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="B60" s="72" t="s">
         <v>151</v>
       </c>
-      <c r="D60" s="73" t="s">
-        <v>157</v>
-      </c>
-      <c r="E60" s="79"/>
-      <c r="F60" s="79"/>
+      <c r="C60" s="72" t="s">
+        <v>153</v>
+      </c>
+      <c r="D60" s="72" t="s">
+        <v>159</v>
+      </c>
+      <c r="E60" s="78"/>
+      <c r="F60" s="78"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="B61" s="72" t="s">
-        <v>146</v>
-      </c>
-      <c r="C61" s="72" t="s">
-        <v>176</v>
-      </c>
-      <c r="D61" s="72" t="s">
-        <v>173</v>
-      </c>
-      <c r="E61" s="79"/>
-      <c r="F61" s="79"/>
+        <v>215</v>
+      </c>
+      <c r="B61" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="C61" s="71" t="s">
+        <v>178</v>
+      </c>
+      <c r="D61" s="71" t="s">
+        <v>175</v>
+      </c>
+      <c r="E61" s="78"/>
+      <c r="F61" s="78"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="B62" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C62" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D62" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E62" s="79"/>
-      <c r="F62" s="79"/>
+        <v>216</v>
+      </c>
+      <c r="B62" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C62" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D62" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E62" s="78"/>
+      <c r="F62" s="78"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="s">
-        <v>215</v>
-      </c>
-      <c r="B63" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="C63" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="D63" s="78" t="s">
-        <v>180</v>
-      </c>
-      <c r="E63" s="79"/>
-      <c r="F63" s="79"/>
+        <v>217</v>
+      </c>
+      <c r="B63" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="C63" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D63" s="77" t="s">
+        <v>182</v>
+      </c>
+      <c r="E63" s="78"/>
+      <c r="F63" s="78"/>
     </row>
     <row r="64">
       <c r="E64" s="42"/>
@@ -10409,138 +10456,138 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="B65" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C65" s="73" t="s">
+        <v>218</v>
+      </c>
+      <c r="B65" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C65" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="D65" s="73" t="s">
+      <c r="D65" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="E65" s="79"/>
-      <c r="F65" s="79"/>
+      <c r="E65" s="78"/>
+      <c r="F65" s="78"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="B66" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C66" s="72" t="s">
-        <v>150</v>
-      </c>
-      <c r="D66" s="72" t="s">
+        <v>220</v>
+      </c>
+      <c r="B66" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C66" s="71" t="s">
+        <v>152</v>
+      </c>
+      <c r="D66" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="E66" s="79"/>
-      <c r="F66" s="79"/>
+      <c r="E66" s="78"/>
+      <c r="F66" s="78"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B67" s="79" t="s">
         <v>219</v>
       </c>
-      <c r="B67" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C67" s="72" t="s">
-        <v>157</v>
-      </c>
-      <c r="D67" s="72" t="s">
+      <c r="C67" s="71" t="s">
+        <v>159</v>
+      </c>
+      <c r="D67" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="E67" s="79"/>
-      <c r="F67" s="79"/>
+      <c r="E67" s="78"/>
+      <c r="F67" s="78"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="B68" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C68" s="71" t="s">
-        <v>221</v>
-      </c>
-      <c r="D68" s="71" t="s">
-        <v>166</v>
-      </c>
-      <c r="E68" s="79"/>
-      <c r="F68" s="79"/>
+        <v>222</v>
+      </c>
+      <c r="B68" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C68" s="70" t="s">
+        <v>223</v>
+      </c>
+      <c r="D68" s="70" t="s">
+        <v>168</v>
+      </c>
+      <c r="E68" s="78"/>
+      <c r="F68" s="78"/>
     </row>
     <row r="69">
-      <c r="B69" s="81"/>
-      <c r="C69" s="82"/>
-      <c r="D69" s="82"/>
+      <c r="B69" s="80"/>
+      <c r="C69" s="81"/>
+      <c r="D69" s="81"/>
       <c r="E69" s="42"/>
       <c r="F69" s="42"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="B70" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C70" s="71" t="s">
-        <v>143</v>
-      </c>
-      <c r="D70" s="71" t="s">
+        <v>224</v>
+      </c>
+      <c r="B70" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C70" s="70" t="s">
+        <v>145</v>
+      </c>
+      <c r="D70" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="E70" s="83"/>
-      <c r="F70" s="83"/>
+      <c r="E70" s="82"/>
+      <c r="F70" s="82"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="B71" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C71" s="77" t="s">
-        <v>224</v>
-      </c>
-      <c r="D71" s="77" t="s">
+        <v>225</v>
+      </c>
+      <c r="B71" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C71" s="76" t="s">
+        <v>226</v>
+      </c>
+      <c r="D71" s="76" t="s">
         <v>53</v>
       </c>
-      <c r="E71" s="83"/>
-      <c r="F71" s="83"/>
+      <c r="E71" s="82"/>
+      <c r="F71" s="82"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="B72" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C72" s="77" t="s">
-        <v>226</v>
-      </c>
-      <c r="D72" s="77" t="s">
+        <v>227</v>
+      </c>
+      <c r="B72" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C72" s="76" t="s">
+        <v>228</v>
+      </c>
+      <c r="D72" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="E72" s="83"/>
-      <c r="F72" s="83"/>
+      <c r="E72" s="82"/>
+      <c r="F72" s="82"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="B73" s="80" t="s">
-        <v>217</v>
-      </c>
-      <c r="C73" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="D73" s="73" t="s">
-        <v>154</v>
-      </c>
-      <c r="E73" s="83"/>
-      <c r="F73" s="83"/>
+        <v>229</v>
+      </c>
+      <c r="B73" s="79" t="s">
+        <v>219</v>
+      </c>
+      <c r="C73" s="72" t="s">
+        <v>175</v>
+      </c>
+      <c r="D73" s="72" t="s">
+        <v>156</v>
+      </c>
+      <c r="E73" s="82"/>
+      <c r="F73" s="82"/>
     </row>
     <row r="74">
       <c r="B74" s="40"/>
@@ -10549,51 +10596,51 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="B75" s="84" t="s">
-        <v>229</v>
-      </c>
-      <c r="C75" s="73"/>
-      <c r="D75" s="73"/>
-      <c r="E75" s="52"/>
-      <c r="F75" s="52"/>
+        <v>230</v>
+      </c>
+      <c r="B75" s="83" t="s">
+        <v>231</v>
+      </c>
+      <c r="C75" s="72"/>
+      <c r="D75" s="72"/>
+      <c r="E75" s="51"/>
+      <c r="F75" s="51"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="B76" s="84" t="s">
-        <v>229</v>
-      </c>
-      <c r="C76" s="72"/>
-      <c r="D76" s="72"/>
-      <c r="E76" s="52"/>
-      <c r="F76" s="52"/>
+        <v>232</v>
+      </c>
+      <c r="B76" s="83" t="s">
+        <v>231</v>
+      </c>
+      <c r="C76" s="71"/>
+      <c r="D76" s="71"/>
+      <c r="E76" s="51"/>
+      <c r="F76" s="51"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B77" s="83" t="s">
         <v>231</v>
       </c>
-      <c r="B77" s="84" t="s">
-        <v>229</v>
-      </c>
-      <c r="C77" s="71"/>
-      <c r="D77" s="71"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="52"/>
+      <c r="C77" s="70"/>
+      <c r="D77" s="70"/>
+      <c r="E77" s="51"/>
+      <c r="F77" s="51"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="B78" s="84" t="s">
-        <v>229</v>
-      </c>
-      <c r="C78" s="77"/>
-      <c r="D78" s="77"/>
-      <c r="E78" s="52"/>
-      <c r="F78" s="52"/>
+        <v>234</v>
+      </c>
+      <c r="B78" s="83" t="s">
+        <v>231</v>
+      </c>
+      <c r="C78" s="76"/>
+      <c r="D78" s="76"/>
+      <c r="E78" s="51"/>
+      <c r="F78" s="51"/>
     </row>
     <row r="79">
       <c r="E79" s="42"/>
@@ -10601,27 +10648,27 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="B80" s="84" t="s">
-        <v>126</v>
-      </c>
-      <c r="C80" s="72"/>
-      <c r="D80" s="85"/>
-      <c r="E80" s="52"/>
-      <c r="F80" s="52"/>
+        <v>235</v>
+      </c>
+      <c r="B80" s="83" t="s">
+        <v>127</v>
+      </c>
+      <c r="C80" s="71"/>
+      <c r="D80" s="84"/>
+      <c r="E80" s="51"/>
+      <c r="F80" s="51"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="B81" s="84" t="s">
-        <v>126</v>
-      </c>
-      <c r="C81" s="77"/>
-      <c r="D81" s="73"/>
-      <c r="E81" s="52"/>
-      <c r="F81" s="52"/>
+        <v>236</v>
+      </c>
+      <c r="B81" s="83" t="s">
+        <v>127</v>
+      </c>
+      <c r="C81" s="76"/>
+      <c r="D81" s="72"/>
+      <c r="E81" s="51"/>
+      <c r="F81" s="51"/>
     </row>
     <row r="82">
       <c r="E82" s="42"/>
@@ -10629,10 +10676,10 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
@@ -10641,10 +10688,10 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
@@ -14331,111 +14378,111 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="85" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" s="55" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>155</v>
+      </c>
+      <c r="E1" s="57" t="s">
+        <v>170</v>
+      </c>
+      <c r="F1" s="58" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="72" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="71" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="C2" s="69" t="s">
+        <v>239</v>
+      </c>
+      <c r="D2" s="86" t="s">
+        <v>240</v>
+      </c>
+      <c r="E2" s="76" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="87" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="72" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="71" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="69">
+        <v>104.0</v>
+      </c>
+      <c r="D3" s="86" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="76" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="87" t="s">
         <v>146</v>
       </c>
-      <c r="C1" s="56" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="57" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="72" t="s">
+        <v>152</v>
+      </c>
+      <c r="B4" s="71" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="86" t="s">
+        <v>168</v>
+      </c>
+      <c r="E4" s="76" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="87" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="72" t="s">
         <v>153</v>
       </c>
-      <c r="E1" s="58" t="s">
-        <v>168</v>
-      </c>
-      <c r="F1" s="59" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="73" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="72" t="s">
-        <v>147</v>
-      </c>
-      <c r="C2" s="70" t="s">
-        <v>237</v>
-      </c>
-      <c r="D2" s="87" t="s">
-        <v>238</v>
-      </c>
-      <c r="E2" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="88" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="73" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" s="72" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="70">
-        <v>104.0</v>
-      </c>
-      <c r="D3" s="87" t="s">
-        <v>154</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="88" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="73" t="s">
-        <v>150</v>
-      </c>
-      <c r="B4" s="72" t="s">
+      <c r="B5" s="71" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="70" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="87" t="s">
-        <v>166</v>
-      </c>
-      <c r="E4" s="77" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="88" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="73" t="s">
-        <v>151</v>
-      </c>
-      <c r="B5" s="72" t="s">
-        <v>176</v>
-      </c>
-      <c r="C5" s="70" t="s">
+      <c r="C5" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="87" t="s">
-        <v>155</v>
-      </c>
-      <c r="E5" s="77" t="s">
-        <v>170</v>
-      </c>
-      <c r="F5" s="88" t="s">
-        <v>162</v>
+      <c r="D5" s="86" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" s="76" t="s">
+        <v>172</v>
+      </c>
+      <c r="F5" s="87" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="73" t="s">
-        <v>157</v>
-      </c>
-      <c r="B6" s="72" t="s">
-        <v>173</v>
+      <c r="A6" s="72" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="71" t="s">
+        <v>175</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>

</xml_diff>

<commit_message>
Dati: risultati semifinali + accoppiamenti finali
- Semifinale: I Cugini-Gli Zebis 8-12 (passa Gli Zebis).
- Semifinale: Bad Boys-Lord&Chri 3-12 (passa Lord&Chri).
- Generate le finali: Finale Gli Zebis-Lord&Chri, 3o/4o I Cugini-Bad Boys.
- Check campo unico: nessuna sovrapposizione di slot.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026.xlsx
+++ b/Resources/Calend Bocce 2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="241">
   <si>
     <t>data e ora</t>
   </si>
@@ -743,7 +743,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -798,6 +798,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -915,7 +921,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1047,34 +1053,34 @@
     <xf borderId="1" fillId="2" fontId="9" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="10" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="11" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="9" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1128,16 +1134,19 @@
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="12" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="12" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -2804,8 +2813,12 @@
       <c r="D85" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="E85" s="51"/>
-      <c r="F85" s="51"/>
+      <c r="E85" s="51">
+        <v>8.0</v>
+      </c>
+      <c r="F85" s="51">
+        <v>12.0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
@@ -2820,8 +2833,12 @@
       <c r="D86" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="E86" s="51"/>
-      <c r="F86" s="51"/>
+      <c r="E86" s="51">
+        <v>3.0</v>
+      </c>
+      <c r="F86" s="51">
+        <v>12.0</v>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="39"/>
@@ -2837,8 +2854,12 @@
       <c r="B88" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="C88" s="48"/>
-      <c r="D88" s="48"/>
+      <c r="C88" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D88" s="48" t="s">
+        <v>53</v>
+      </c>
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
     </row>
@@ -2849,8 +2870,12 @@
       <c r="B89" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="C89" s="48"/>
-      <c r="D89" s="48"/>
+      <c r="C89" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="D89" s="48" t="s">
+        <v>40</v>
+      </c>
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
     </row>
@@ -10603,8 +10628,8 @@
       </c>
       <c r="C75" s="72"/>
       <c r="D75" s="72"/>
-      <c r="E75" s="51"/>
-      <c r="F75" s="51"/>
+      <c r="E75" s="84"/>
+      <c r="F75" s="84"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
@@ -10615,8 +10640,8 @@
       </c>
       <c r="C76" s="71"/>
       <c r="D76" s="71"/>
-      <c r="E76" s="51"/>
-      <c r="F76" s="51"/>
+      <c r="E76" s="84"/>
+      <c r="F76" s="84"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
@@ -10627,8 +10652,8 @@
       </c>
       <c r="C77" s="70"/>
       <c r="D77" s="70"/>
-      <c r="E77" s="51"/>
-      <c r="F77" s="51"/>
+      <c r="E77" s="84"/>
+      <c r="F77" s="84"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
@@ -10639,8 +10664,8 @@
       </c>
       <c r="C78" s="76"/>
       <c r="D78" s="76"/>
-      <c r="E78" s="51"/>
-      <c r="F78" s="51"/>
+      <c r="E78" s="84"/>
+      <c r="F78" s="84"/>
     </row>
     <row r="79">
       <c r="E79" s="42"/>
@@ -10654,9 +10679,9 @@
         <v>127</v>
       </c>
       <c r="C80" s="71"/>
-      <c r="D80" s="84"/>
-      <c r="E80" s="51"/>
-      <c r="F80" s="51"/>
+      <c r="D80" s="85"/>
+      <c r="E80" s="84"/>
+      <c r="F80" s="84"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
@@ -10667,8 +10692,8 @@
       </c>
       <c r="C81" s="76"/>
       <c r="D81" s="72"/>
-      <c r="E81" s="51"/>
-      <c r="F81" s="51"/>
+      <c r="E81" s="84"/>
+      <c r="F81" s="84"/>
     </row>
     <row r="82">
       <c r="E82" s="42"/>
@@ -14378,7 +14403,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="86" t="s">
         <v>151</v>
       </c>
       <c r="B1" s="54" t="s">
@@ -14407,13 +14432,13 @@
       <c r="C2" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="D2" s="86" t="s">
+      <c r="D2" s="87" t="s">
         <v>240</v>
       </c>
       <c r="E2" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="87" t="s">
+      <c r="F2" s="88" t="s">
         <v>145</v>
       </c>
     </row>
@@ -14427,13 +14452,13 @@
       <c r="C3" s="69">
         <v>104.0</v>
       </c>
-      <c r="D3" s="86" t="s">
+      <c r="D3" s="87" t="s">
         <v>156</v>
       </c>
       <c r="E3" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="87" t="s">
+      <c r="F3" s="88" t="s">
         <v>146</v>
       </c>
     </row>
@@ -14447,13 +14472,13 @@
       <c r="C4" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="86" t="s">
+      <c r="D4" s="87" t="s">
         <v>168</v>
       </c>
       <c r="E4" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="87" t="s">
+      <c r="F4" s="88" t="s">
         <v>37</v>
       </c>
     </row>
@@ -14467,13 +14492,13 @@
       <c r="C5" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="86" t="s">
+      <c r="D5" s="87" t="s">
         <v>157</v>
       </c>
       <c r="E5" s="76" t="s">
         <v>172</v>
       </c>
-      <c r="F5" s="87" t="s">
+      <c r="F5" s="88" t="s">
         <v>164</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dati: risultati delle finali - Lord&Chri campione 2026
- Finale: Gli Zebis - Lord&Chri 4-13
- Finale 3/4 posto: I Cugini - Bad Boys 12-0
- Check campo unico: nessuna sovrapposizione

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026.xlsx
+++ b/Resources/Calend Bocce 2026.xlsx
@@ -2860,8 +2860,12 @@
       <c r="D88" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
+      <c r="E88" s="5">
+        <v>12.0</v>
+      </c>
+      <c r="F88" s="5">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
@@ -2876,8 +2880,12 @@
       <c r="D89" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
+      <c r="E89" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="F89" s="5">
+        <v>13.0</v>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="39"/>

</xml_diff>